<commit_message>
MS #158: resolve Coffeeville + Leland (both Consolidated/Elected) — classification complete
</commit_message>
<xml_diff>
--- a/reference/MS Rolling Audit/MS_Municipalities.xlsx
+++ b/reference/MS Rolling Audit/MS_Municipalities.xlsx
@@ -19814,7 +19814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="8" min="1" max="1"/>
@@ -20014,27 +20014,54 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Classification pass completed for the 66 Needs Research districts (issue #158), from official sources (OSA audit Note 1s, district/city official pages, Miss. Code §37-7-203 incl. subsections (3) Jackson, (4) Moss Point, (5) Newton). Results: 12 Elected, 11 Mixed (appointed majority + elected added-territory seats), 35 Appointed (incl. statutory-default), 8 Unresolved carried forward with conflicts documented (Coffeeville, Leland, and 6 type-unresolved districts whose audits evidence seating). Okolona moved to Deferred (District of Transformation, board abolished 2025-11-14) and Yazoo City flagged Deferred (board suspended, ASD takeover). Spot-checks by Boone: §37-7-203(4)/(5) read firsthand; Alcorn, Grenada, and South Panola audit language verified against the PDFs.</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>School Districts, Status Log</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>MS Office of the State Auditor audits; Miss. Code §37-7-203; district/city official sites</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Boone</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Resolved the last two Unresolved districts (issue #158) on evidence supplied by Walter and verified the same day: Coffeeville = Consolidated / Elected (2025 district board agenda records trustees 're-elected'; McLean-Robinson v. Coffeeville Consolidated School District, N.D. Miss. 2025, styles it CCSD; the FY2024/FY2025 audit 'city selects a majority' language is treated as boilerplate error) and Leland = Consolidated / Elected (Washington County Election Commission official recapitulations show Leland School Board Trustee district elections in 2013, 2020, and 2023; the 2023 District 1 winner appears on the district's current roster). Classification is now complete for all 144 districts: 91 Elected, 11 Mixed, 36 Appointed, 6 charter out of scope; 4 deferred.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>School Districts, Status Log</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Coffeeville SD board agenda (2025); N.D. Miss. No. 3:2024cv00048 Doc. 49; Washington County Election Commission recapitulations (2013, 2020, 2023)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>Boone</t>
         </is>
@@ -20135,7 +20162,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F2" s="8" t="inlineStr">
@@ -20180,7 +20207,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F3" s="8" t="inlineStr">
@@ -20304,7 +20331,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -20390,7 +20417,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -20435,7 +20462,7 @@
           <t>Appointed</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -20521,7 +20548,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -20566,7 +20593,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -20611,7 +20638,7 @@
           <t>Appointed</t>
         </is>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -20697,7 +20724,7 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -20944,7 +20971,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E21" t="n">
+      <c r="E21" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -20985,7 +21012,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E22" t="n">
+      <c r="E22" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -21030,7 +21057,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E23" t="n">
+      <c r="E23" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -21108,20 +21135,20 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Unresolved</t>
+          <t>Consolidated</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>Unresolved</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
+          <t>Elected</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>Official sources conflict. The FY2016 OSA-hosted audit describes a primary government governed by a five member board with each member elected by the citizens of each defined county district, and a 1973 federal caption styles it Coffeeville Consolidated School District; the FY2024 and FY2025 audits instead state the district is a related organization of the city of Coffeeville since the city's governing authority selects a majority of the board. County-administered November trustee elections from five positions are documented through 2020, but the conflict between the audits could not be resolved from official sources. [https://www.osa.ms.gov/sites/default/files/osa/files/reports/25s2025%20Coffeeville%20School%20District-cpa.pdf]</t>
+          <t>Resolved 2026-10-16 (evidence supplied by Walter, verified by Boone): the district's 2025 board agenda records trustees as 're-elected' with oaths of office (incl. a 4th Ward member 'elected'), and McLean-Robinson v. Coffeeville Consolidated School District, No. 3:2024cv00048, Doc. 49 (N.D. Miss. 2025), styles the district 'Coffeeville Consolidated School District (CCSD)' throughout — consistent with the FY2016 OSA audit's elected-board language. [https://content.myconnectsuite.com/api/documents/16bb40fd09ed4039b92de38b07622127.pdf ; https://law.justia.com/cases/federal/district-courts/mississippi/msndce/3:2024cv00048/48951/49/]</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
@@ -21131,12 +21158,12 @@
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>Needs Research — follow-up</t>
+          <t>Classified — ready for roster pass</t>
         </is>
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>Type unresolved — classification pass (Code provisos + local acts)</t>
+          <t>Type unresolved — classification pass (Code provisos + local acts) RESOLVED: Consolidated / Elected. The FY2024 and FY2025 OSA audits' 'city selects a majority' Note 1 language is treated as GASB boilerplate error — the same sentence appears for districts known to be fully appointed (Corinth) and is outweighed by the 2025 agenda, the 2025 federal caption, the FY2016 audit, and county trustee elections documented through 2020.</t>
         </is>
       </c>
     </row>
@@ -21161,7 +21188,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E26" t="n">
+      <c r="E26" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -21206,7 +21233,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E27" t="n">
+      <c r="E27" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -21288,7 +21315,7 @@
           <t>Appointed</t>
         </is>
       </c>
-      <c r="E29" t="n">
+      <c r="E29" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F29" s="8" t="inlineStr">
@@ -21419,7 +21446,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E32" t="n">
+      <c r="E32" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F32" s="8" t="inlineStr">
@@ -21505,7 +21532,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E34" t="n">
+      <c r="E34" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F34" s="8" t="inlineStr">
@@ -21550,7 +21577,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E35" t="n">
+      <c r="E35" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F35" s="8" t="inlineStr">
@@ -21591,7 +21618,7 @@
           <t>Appointed</t>
         </is>
       </c>
-      <c r="E36" t="n">
+      <c r="E36" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F36" s="8" t="inlineStr">
@@ -21796,7 +21823,7 @@
           <t>Appointed</t>
         </is>
       </c>
-      <c r="E41" t="n">
+      <c r="E41" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F41" s="8" t="inlineStr">
@@ -21882,7 +21909,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E43" t="n">
+      <c r="E43" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F43" s="8" t="inlineStr">
@@ -21927,7 +21954,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E44" t="n">
+      <c r="E44" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -22054,7 +22081,7 @@
           <t>Appointed</t>
         </is>
       </c>
-      <c r="E47" t="n">
+      <c r="E47" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F47" s="8" t="inlineStr">
@@ -22099,7 +22126,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E48" t="n">
+      <c r="E48" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F48" s="8" t="inlineStr">
@@ -22185,7 +22212,7 @@
           <t>Appointed</t>
         </is>
       </c>
-      <c r="E50" t="n">
+      <c r="E50" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F50" s="8" t="inlineStr">
@@ -22230,7 +22257,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E51" t="n">
+      <c r="E51" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F51" s="8" t="inlineStr">
@@ -22443,7 +22470,7 @@
           <t>Appointed</t>
         </is>
       </c>
-      <c r="E56" t="n">
+      <c r="E56" s="8" t="n">
         <v>7</v>
       </c>
       <c r="F56" s="8" t="inlineStr">
@@ -22728,7 +22755,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E63" t="n">
+      <c r="E63" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F63" s="8" t="inlineStr">
@@ -22896,7 +22923,7 @@
           <t>Appointed</t>
         </is>
       </c>
-      <c r="E67" t="n">
+      <c r="E67" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F67" s="8" t="inlineStr">
@@ -23056,20 +23083,20 @@
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>Unresolved</t>
+          <t>Consolidated</t>
         </is>
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>Unresolved</t>
-        </is>
-      </c>
-      <c r="E71" t="n">
+          <t>Elected</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F71" s="8" t="inlineStr">
         <is>
-          <t>Checked the district website, Title 37 Ch. 7, the unenacted 2014–2016 Hollandale–Leland consolidation bills, MDE, and OSA audits: sources conflict and none names the legal type — a 2013 MDE agenda lists 'Leland Consolidated School District' by name only, while the FY2023 OSA audit says the City of Leland's governing authority selects a majority of the board and levies its taxes (a municipal-separate pattern); the audit does establish five board members. A district-specific act or official type listing is still needed. [https://www.osa.ms.gov/sites/default/files/osa/files/reports/23s2023%20Leland%20School%20District-cpa.pdf]</t>
+          <t>Resolved 2026-10-16 (evidence supplied by Walter): the Washington County Election Commission's official November 7, 2023 general-election recapitulation contains a 'LELAND SCHOOL BOARD TRUSTEE DIST 1' contest (Patansy Miller Hampton; Joe Ann Williams), and Williams appears as the District 1 trustee on the district's own current board roster; county records also show Trustee District 1 (Nov. 5, 2013) and District 5 (Nov. 3, 2020) elections. Consistent with the 2013 MDE agenda naming it 'Leland Consolidated School District.'</t>
         </is>
       </c>
       <c r="G71" s="8" t="inlineStr">
@@ -23079,12 +23106,12 @@
       </c>
       <c r="H71" s="8" t="inlineStr">
         <is>
-          <t>Needs Research — follow-up</t>
+          <t>Classified — ready for roster pass</t>
         </is>
       </c>
       <c r="I71" s="8" t="inlineStr">
         <is>
-          <t>Type unresolved — classification pass (Code provisos + local acts)</t>
+          <t>Type unresolved — classification pass (Code provisos + local acts) RESOLVED: Consolidated / Elected on county-run trustee-district elections (2013, 2020, 2023). The FY2023 OSA audit's city-selects-a-majority language is outweighed by the official election records.</t>
         </is>
       </c>
     </row>
@@ -23150,7 +23177,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E73" t="n">
+      <c r="E73" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F73" s="8" t="inlineStr">
@@ -23195,7 +23222,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E74" t="n">
+      <c r="E74" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F74" s="8" t="inlineStr">
@@ -23400,7 +23427,7 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="E79" t="n">
+      <c r="E79" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F79" s="8" t="inlineStr">
@@ -23441,7 +23468,7 @@
           <t>Appointed</t>
         </is>
       </c>
-      <c r="E80" t="n">
+      <c r="E80" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F80" s="8" t="inlineStr">
@@ -23565,7 +23592,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E83" t="n">
+      <c r="E83" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F83" s="8" t="inlineStr">
@@ -23610,7 +23637,7 @@
           <t>Appointed</t>
         </is>
       </c>
-      <c r="E84" t="n">
+      <c r="E84" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F84" s="8" t="inlineStr">
@@ -23696,7 +23723,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E86" t="n">
+      <c r="E86" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F86" s="8" t="inlineStr">
@@ -23741,7 +23768,7 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="E87" t="n">
+      <c r="E87" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F87" s="8" t="inlineStr">
@@ -23827,7 +23854,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E89" t="n">
+      <c r="E89" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F89" s="8" t="inlineStr">
@@ -23909,7 +23936,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E91" t="n">
+      <c r="E91" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F91" s="8" t="inlineStr">
@@ -24081,7 +24108,7 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="E95" t="n">
+      <c r="E95" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F95" s="8" t="inlineStr">
@@ -24126,7 +24153,7 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="E96" t="n">
+      <c r="E96" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F96" s="8" t="inlineStr">
@@ -24171,7 +24198,7 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="E97" t="n">
+      <c r="E97" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F97" s="8" t="inlineStr">
@@ -24216,7 +24243,7 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="E98" t="n">
+      <c r="E98" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F98" s="8" t="inlineStr">
@@ -24261,7 +24288,7 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="E99" t="n">
+      <c r="E99" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F99" s="8" t="inlineStr">
@@ -24306,7 +24333,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E100" t="n">
+      <c r="E100" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F100" s="8" t="inlineStr">
@@ -24433,7 +24460,7 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="E103" t="n">
+      <c r="E103" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F103" s="8" t="inlineStr">
@@ -24478,7 +24505,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E104" t="n">
+      <c r="E104" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F104" s="8" t="inlineStr">
@@ -24523,7 +24550,7 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="E105" t="n">
+      <c r="E105" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F105" s="8" t="inlineStr">
@@ -24568,7 +24595,7 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="E106" t="n">
+      <c r="E106" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F106" s="8" t="inlineStr">
@@ -24654,7 +24681,7 @@
           <t>Appointed</t>
         </is>
       </c>
-      <c r="E108" t="n">
+      <c r="E108" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F108" s="8" t="inlineStr">
@@ -24781,7 +24808,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E111" t="n">
+      <c r="E111" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F111" s="8" t="inlineStr">
@@ -24905,7 +24932,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E114" t="n">
+      <c r="E114" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F114" s="8" t="inlineStr">
@@ -24991,7 +25018,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E116" t="n">
+      <c r="E116" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F116" s="8" t="inlineStr">
@@ -25114,7 +25141,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E119" t="n">
+      <c r="E119" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F119" s="8" t="inlineStr">
@@ -25159,7 +25186,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E120" t="n">
+      <c r="E120" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F120" s="8" t="inlineStr">
@@ -25204,7 +25231,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E121" t="n">
+      <c r="E121" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F121" s="8" t="inlineStr">
@@ -25249,7 +25276,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E122" t="n">
+      <c r="E122" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F122" s="8" t="inlineStr">
@@ -25458,7 +25485,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E127" t="n">
+      <c r="E127" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F127" s="8" t="inlineStr">
@@ -25540,7 +25567,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E129" t="n">
+      <c r="E129" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F129" s="8" t="inlineStr">
@@ -25626,7 +25653,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E131" t="n">
+      <c r="E131" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F131" s="8" t="inlineStr">
@@ -25671,7 +25698,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E132" t="n">
+      <c r="E132" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F132" s="8" t="inlineStr">
@@ -25757,7 +25784,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E134" t="n">
+      <c r="E134" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F134" s="8" t="inlineStr">
@@ -26048,7 +26075,7 @@
           <t>Elected</t>
         </is>
       </c>
-      <c r="E141" t="n">
+      <c r="E141" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F141" s="8" t="inlineStr">
@@ -26175,7 +26202,7 @@
           <t>Appointed (statutory default §37-7-203(1))</t>
         </is>
       </c>
-      <c r="E144" t="n">
+      <c r="E144" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F144" s="8" t="inlineStr">

</xml_diff>

<commit_message>
MS #158: roster-pass sheet update (68 minted, 27 held, Humphreys + Wilkinson deferred as Districts of Transformation)
</commit_message>
<xml_diff>
--- a/reference/MS Rolling Audit/MS_Municipalities.xlsx
+++ b/reference/MS Rolling Audit/MS_Municipalities.xlsx
@@ -20041,27 +20041,27 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Resolved the last two Unresolved districts (issue #158) on evidence supplied by Walter and verified the same day: Coffeeville = Consolidated / Elected (2025 district board agenda records trustees 're-elected'; McLean-Robinson v. Coffeeville Consolidated School District, N.D. Miss. 2025, styles it CCSD; the FY2024/FY2025 audit 'city selects a majority' language is treated as boilerplate error) and Leland = Consolidated / Elected (Washington County Election Commission official recapitulations show Leland School Board Trustee district elections in 2013, 2020, and 2023; the 2023 District 1 winner appears on the district's current roster). Classification is now complete for all 144 districts: 91 Elected, 11 Mixed, 36 Appointed, 6 charter out of scope; 4 deferred.</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>School Districts, Status Log</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>Coffeeville SD board agenda (2025); N.D. Miss. No. 3:2024cv00048 Doc. 49; Washington County Election Commission recapitulations (2013, 2020, 2023)</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Boone</t>
         </is>
@@ -20217,12 +20217,12 @@
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.alcornschools.org/o/alcorn-school-district/page/school-board</t>
         </is>
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I3" s="8" t="inlineStr">
@@ -20300,12 +20300,12 @@
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.amite.k12.ms.us/schoolboard</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr"/>
@@ -20386,12 +20386,12 @@
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.attala.k12.ms.us/apps/pages/index.jsp?uREC_ID=4428302&amp;type=d&amp;pREC_ID=2665861</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I7" s="8" t="inlineStr"/>
@@ -20517,12 +20517,12 @@
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.benton.k12.ms.us/boe</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr"/>
@@ -20693,12 +20693,12 @@
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.calhounk12.com/schoolboard</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr"/>
@@ -20734,17 +20734,17 @@
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.cantonschools.net/our-district/about-our-district/board-members</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Roster held</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>Type unresolved — classification pass (Code provisos + local acts)</t>
+          <t>Held - roster lists 5 trustees but publishes no per-member elected/appointed labels for this Mixed board, and the page may lag current membership; needs a source labeling each member.</t>
         </is>
       </c>
     </row>
@@ -20779,12 +20779,12 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.ccsd.ms/boardmembers</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I16" s="8" t="inlineStr"/>
@@ -20820,12 +20820,12 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.chickasaw.k12.ms.us/page/board-of-trustees</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr"/>
@@ -20861,12 +20861,12 @@
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.choctaw.k12.ms.us/o/choctawsd/page/school-board</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr"/>
@@ -20902,12 +20902,12 @@
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.claiborne.k12.ms.us/board-of-education/school-board</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr"/>
@@ -21112,12 +21112,12 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.coahomak12.org/about/administration</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I24" s="8" t="inlineStr"/>
@@ -21153,17 +21153,17 @@
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.coffeevilleschools.org/boardmembers</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Roster held</t>
         </is>
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>Type unresolved — classification pass (Code provisos + local acts) RESOLVED: Consolidated / Elected. The FY2024 and FY2025 OSA audits' 'city selects a majority' Note 1 language is treated as GASB boilerplate error — the same sentence appears for districts known to be fully appointed (Corinth) and is outweighed by the 2025 agenda, the 2025 federal caption, the FY2016 audit, and county trustee elections documented through 2020.</t>
+          <t>Held - district board page names only 4 of 5 trustees; fifth member not named in any official source found.</t>
         </is>
       </c>
     </row>
@@ -21289,10 +21289,14 @@
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I28" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>Held - district site (www.copiah.ms) unreachable during capture; no official roster located.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
@@ -21370,12 +21374,12 @@
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://covingtoncountyschools.org/en-US/school-board-240263f6/board-members-1431ea49</t>
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I30" s="8" t="inlineStr"/>
@@ -21456,12 +21460,12 @@
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.eastjasper.k12.ms.us/o/east-jasper/page/board-of-education</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I32" s="8" t="inlineStr">
@@ -21501,12 +21505,12 @@
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.etsd.k12.ms.us/schoolboard</t>
         </is>
       </c>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I33" s="8" t="inlineStr"/>
@@ -21542,17 +21546,17 @@
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.esd.k12.ms.us/en-US/school-board-3242472b</t>
         </is>
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Roster held</t>
         </is>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>Type unresolved — classification pass (Code provisos + local acts)</t>
+          <t>Held - only published roster is headed '2022-2023 School Year'; may be stale.</t>
         </is>
       </c>
     </row>
@@ -21669,12 +21673,12 @@
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.fcsd.us/boardmembers</t>
         </is>
       </c>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I37" s="8" t="inlineStr"/>
@@ -21710,12 +21714,12 @@
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.franklincountyschoolsms.com/members</t>
         </is>
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I38" s="8" t="inlineStr"/>
@@ -21751,12 +21755,12 @@
       </c>
       <c r="G39" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.gcsd.us/school-board</t>
         </is>
       </c>
       <c r="H39" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I39" s="8" t="inlineStr"/>
@@ -21797,10 +21801,14 @@
       </c>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I40" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>Held - district site returns no readable board page; no official roster located.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
@@ -21878,12 +21886,12 @@
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.glcsd.org/board</t>
         </is>
       </c>
       <c r="H42" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I42" s="8" t="inlineStr"/>
@@ -21919,12 +21927,12 @@
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.grenadak12.com/about-us/school-board</t>
         </is>
       </c>
       <c r="H43" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I43" s="8" t="inlineStr">
@@ -22009,12 +22017,12 @@
       </c>
       <c r="G45" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.hancockschools.net/school-board</t>
         </is>
       </c>
       <c r="H45" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I45" s="8" t="inlineStr"/>
@@ -22050,12 +22058,12 @@
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.harrison.k12.ms.us/22309_3</t>
         </is>
       </c>
       <c r="H46" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I46" s="8" t="inlineStr"/>
@@ -22181,12 +22189,12 @@
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://files-backend.assets.thrillshare.com/documents/asset/uploaded_file/4080/Hcsd/00de5838-c25b-42cf-a052-7a34899701e7/July_2__2025_-_Superintendent___Chief_Learner_.pdf?disposition=inline</t>
         </is>
       </c>
       <c r="H49" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I49" s="8" t="inlineStr"/>
@@ -22362,10 +22370,14 @@
       </c>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I53" s="8" t="inlineStr"/>
+          <t>Deferred - District of Transformation</t>
+        </is>
+      </c>
+      <c r="I53" s="8" t="inlineStr">
+        <is>
+          <t>District of Transformation: the local board is not functioning; the district is state-led under MDE (Humphreys: district's official Jan. 23, 2025 Q&amp;A states Districts of Transformation have no school board; Wilkinson: MDE news release, Jan. 15, 2026). Deferred with the other Transformation districts.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
@@ -22398,12 +22410,12 @@
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://resources.finalsite.net/images/v1762413621/itawambacsdcom/lao2tjusznwnnpg9srhz/2025-2026ICSDDropoutPreventionPlan.pdf</t>
         </is>
       </c>
       <c r="H54" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I54" s="8" t="inlineStr"/>
@@ -22439,12 +22451,12 @@
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>http://www.jcsd.ms/our-district/school-board/board-member-bio</t>
         </is>
       </c>
       <c r="H55" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I55" s="8" t="inlineStr"/>
@@ -22525,15 +22537,19 @@
       </c>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>http://www.jcpsd.net/schoolboard</t>
         </is>
       </c>
       <c r="H57" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I57" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I57" s="8" t="inlineStr">
+        <is>
+          <t>Held - official board page names only 3 of 5 members.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
@@ -22566,12 +22582,12 @@
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://resources.finalsite.net/images/v1758644273/jdcsdcom/zol28wg8npyoxcj64t01/ElementaryHandbook2025-20268.pdf</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I58" s="8" t="inlineStr"/>
@@ -22683,12 +22699,12 @@
       </c>
       <c r="G61" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.jones.k12.ms.us/en-US/school-board-members-a198f9dd</t>
         </is>
       </c>
       <c r="H61" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I61" s="8" t="inlineStr"/>
@@ -22724,12 +22740,12 @@
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.kempercountyschools.org/school-board</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I62" s="8" t="inlineStr"/>
@@ -22810,12 +22826,12 @@
       </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://core-docs.s3.us-east-1.amazonaws.com/documents/asset/uploaded_file/4476/LCSD/4147712/2025StudentHanbook.pdf</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I64" s="8" t="inlineStr"/>
@@ -22851,15 +22867,19 @@
       </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://lamarcountyschools.org/school-board</t>
         </is>
       </c>
       <c r="H65" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I65" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I65" s="8" t="inlineStr">
+        <is>
+          <t>Held - official board page names 4 of 5 members; District D shown as an unnamed placeholder.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
@@ -22892,12 +22912,12 @@
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>http://www.lauderdale.k12.ms.us/apps/pages/index.jsp?uREC_ID=1543366&amp;type=d&amp;pREC_ID=1670838</t>
         </is>
       </c>
       <c r="H66" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I66" s="8" t="inlineStr"/>
@@ -22978,12 +22998,12 @@
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://lawcosd.org/52820_3</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I68" s="8" t="inlineStr"/>
@@ -23019,12 +23039,12 @@
       </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://irp.cdn-website.com/61f020bd/files/uploaded/25-26+LCSD+Student+Parent+Handbook+Updated+07222025-B.pdf</t>
         </is>
       </c>
       <c r="H69" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I69" s="8" t="inlineStr"/>
@@ -23060,12 +23080,12 @@
       </c>
       <c r="G70" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>http://www.leecountyschools.us/page/school-board</t>
         </is>
       </c>
       <c r="H70" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I70" s="8" t="inlineStr"/>
@@ -23101,12 +23121,12 @@
       </c>
       <c r="G71" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.lelandk12.org/members</t>
         </is>
       </c>
       <c r="H71" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I71" s="8" t="inlineStr">
@@ -23146,12 +23166,12 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://lcsd.k12.ms.us/apps/news/article/1575384</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I72" s="8" t="inlineStr"/>
@@ -23232,12 +23252,12 @@
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.louisville.k12.ms.us/boardmembers</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I74" s="8" t="inlineStr"/>
@@ -23273,12 +23293,12 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.lowndes.k12.ms.us/parents/files/documents/Handbooks/STUDENT HANDBOOK 26-27- Revised 9-23-26.pdf</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I75" s="8" t="inlineStr"/>
@@ -23314,12 +23334,12 @@
       </c>
       <c r="G76" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://resources.finalsite.net/images/v1762369097/madisonschoolscom/cpxg29tkgmkj451x7uze/2025-2026StudentHandbook-110525.pdf</t>
         </is>
       </c>
       <c r="H76" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I76" s="8" t="inlineStr"/>
@@ -23355,12 +23375,12 @@
       </c>
       <c r="G77" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.marionk12.org/schoolboard</t>
         </is>
       </c>
       <c r="H77" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I77" s="8" t="inlineStr"/>
@@ -23396,15 +23416,19 @@
       </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.marshallcountysd.org/article/909674</t>
         </is>
       </c>
       <c r="H78" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I78" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I78" s="8" t="inlineStr">
+        <is>
+          <t>Held - newest official roster found is a district article dated Nov 15, 2022; may be stale.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
@@ -23437,12 +23461,12 @@
       </c>
       <c r="G79" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>http://www.mccomb.k12.ms.us/apps/pages/index.jsp?uREC_ID=367706&amp;type=d&amp;pREC_ID=823302</t>
         </is>
       </c>
       <c r="H79" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I79" s="8" t="inlineStr"/>
@@ -23561,12 +23585,12 @@
       </c>
       <c r="G82" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.mcsd.us/about-mcsd/school_board</t>
         </is>
       </c>
       <c r="H82" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I82" s="8" t="inlineStr"/>
@@ -23602,12 +23626,12 @@
       </c>
       <c r="G83" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.mpsdnow.org/leadership/school-board</t>
         </is>
       </c>
       <c r="H83" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I83" s="8" t="inlineStr">
@@ -23692,15 +23716,19 @@
       </c>
       <c r="G85" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://files.smartsites.parentsquare.com/5429/employee_handbook_2025-2026_for_website.pdf</t>
         </is>
       </c>
       <c r="H85" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I85" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I85" s="8" t="inlineStr">
+        <is>
+          <t>Held - district 2025-26 handbook and county supervisors page conflict on the District Two member (Nicholson vs. Butler); needs verification.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
@@ -23733,12 +23761,12 @@
       </c>
       <c r="G86" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.nettletonschools.com/page/school-board</t>
         </is>
       </c>
       <c r="H86" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I86" s="8" t="inlineStr">
@@ -23778,17 +23806,17 @@
       </c>
       <c r="G87" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.newalbanyschools.us/about-us/</t>
         </is>
       </c>
       <c r="H87" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Roster held</t>
         </is>
       </c>
       <c r="I87" s="8" t="inlineStr">
         <is>
-          <t>Type unresolved — classification pass (Code provisos + local acts)</t>
+          <t>Held - Mixed board; district page lists all five trustees with no elected/appointed labels; needs a labeling source.</t>
         </is>
       </c>
     </row>
@@ -23823,12 +23851,12 @@
       </c>
       <c r="G88" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.newton.k12.ms.us/69270_2</t>
         </is>
       </c>
       <c r="H88" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I88" s="8" t="inlineStr"/>
@@ -23864,12 +23892,12 @@
       </c>
       <c r="G89" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.nmsd.us/fs/resource-manager/view/3e4685a1-4088-4987-b89a-b244f1dc7978</t>
         </is>
       </c>
       <c r="H89" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I89" s="8" t="inlineStr"/>
@@ -23905,15 +23933,19 @@
       </c>
       <c r="G90" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://campussuite-storage.s3.amazonaws.com/prod/1559046/e9a18732-f28b-11ea-8684-1281cd704e31/2689248/a607479c-7513-11ee-8e76-0a58a9feac02/file/2023%20-2024%20Student%20Handbook%20.pdf</t>
         </is>
       </c>
       <c r="H90" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I90" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I90" s="8" t="inlineStr">
+        <is>
+          <t>Held - newest roster located may be stale (district board page publishes agendas only).</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
@@ -23946,12 +23978,12 @@
       </c>
       <c r="G91" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.northpanolaschools.org/meet-the-members</t>
         </is>
       </c>
       <c r="H91" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I91" s="8" t="inlineStr">
@@ -23991,12 +24023,12 @@
       </c>
       <c r="G92" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://npsd.k12.ms.us/en-US/school-board-of-trustees-6648daa9</t>
         </is>
       </c>
       <c r="H92" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I92" s="8" t="inlineStr"/>
@@ -24032,12 +24064,12 @@
       </c>
       <c r="G93" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.northtippah.org/about-us/administration</t>
         </is>
       </c>
       <c r="H93" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I93" s="8" t="inlineStr"/>
@@ -24118,17 +24150,17 @@
       </c>
       <c r="G95" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.ossdms.org/discoverossd/school-board-policies</t>
         </is>
       </c>
       <c r="H95" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Roster held</t>
         </is>
       </c>
       <c r="I95" s="8" t="inlineStr">
         <is>
-          <t>Type unresolved — classification pass (Code provisos + local acts)</t>
+          <t>Held - Mixed board; district page gives no per-member elected/appointed labels; needs a labeling source.</t>
         </is>
       </c>
     </row>
@@ -24208,17 +24240,17 @@
       </c>
       <c r="G97" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.oxfordsd.org/school-board/board-members</t>
         </is>
       </c>
       <c r="H97" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Roster held</t>
         </is>
       </c>
       <c r="I97" s="8" t="inlineStr">
         <is>
-          <t>Type unresolved — classification pass (Code provisos + local acts)</t>
+          <t>Held - official Board Members page lists only 4 of 5 members.</t>
         </is>
       </c>
     </row>
@@ -24253,12 +24285,12 @@
       </c>
       <c r="G98" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.pgsd.ms/219711_3</t>
         </is>
       </c>
       <c r="H98" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I98" s="8" t="inlineStr">
@@ -24298,17 +24330,17 @@
       </c>
       <c r="G99" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.pc.k12.ms.us/apps/pages/index.jsp?uREC_ID=1196820&amp;type=d&amp;pREC_ID=1438559</t>
         </is>
       </c>
       <c r="H99" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Roster held</t>
         </is>
       </c>
       <c r="I99" s="8" t="inlineStr">
         <is>
-          <t>Type unresolved — classification pass (Code provisos + local acts)</t>
+          <t>Held - Mixed board; district page gives no per-member elected/appointed labels; needs a labeling source.</t>
         </is>
       </c>
     </row>
@@ -24388,12 +24420,12 @@
       </c>
       <c r="G101" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.prc.k12.ms.us/school-board</t>
         </is>
       </c>
       <c r="H101" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I101" s="8" t="inlineStr"/>
@@ -24429,12 +24461,12 @@
       </c>
       <c r="G102" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://pcsdms.com/our-district123/board-of-education</t>
         </is>
       </c>
       <c r="H102" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I102" s="8" t="inlineStr"/>
@@ -24470,12 +24502,12 @@
       </c>
       <c r="G103" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.petalschools.com/our-district/board-of-trustees</t>
         </is>
       </c>
       <c r="H103" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I103" s="8" t="inlineStr">
@@ -24560,17 +24592,17 @@
       </c>
       <c r="G105" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.picayuneschools.org/board-of-trustees</t>
         </is>
       </c>
       <c r="H105" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Roster held</t>
         </is>
       </c>
       <c r="I105" s="8" t="inlineStr">
         <is>
-          <t>Type unresolved — classification pass (Code provisos + local acts)</t>
+          <t>Held - Mixed board; district page gives no per-member elected/appointed labels; needs a labeling source.</t>
         </is>
       </c>
     </row>
@@ -24605,17 +24637,17 @@
       </c>
       <c r="G106" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.pontotoc.school/apps/pages/index.jsp?uREC_ID=2107734&amp;type=d&amp;pREC_ID=2147975</t>
         </is>
       </c>
       <c r="H106" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Roster held</t>
         </is>
       </c>
       <c r="I106" s="8" t="inlineStr">
         <is>
-          <t>Type unresolved — classification pass (Code provisos + local acts)</t>
+          <t>Held - Mixed board; district page gives no per-member elected/appointed labels; needs a labeling source.</t>
         </is>
       </c>
     </row>
@@ -24650,12 +24682,12 @@
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://files-backend.assets.thrillshare.com/documents/asset/uploaded_file/3854/Pcsd/506a880c-2a14-423e-8d70-12655a8f990c/PCSD_Alternative_Handbook_25-26.pdf?disposition=inline</t>
         </is>
       </c>
       <c r="H107" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I107" s="8" t="inlineStr"/>
@@ -24736,12 +24768,12 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.prentisscountyschools.com/school-board</t>
         </is>
       </c>
       <c r="H109" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I109" s="8" t="inlineStr"/>
@@ -24777,12 +24809,12 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.qcschools.com/about/board-of-trustees</t>
         </is>
       </c>
       <c r="H110" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I110" s="8" t="inlineStr"/>
@@ -24818,12 +24850,12 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://campussuite-storage.s3.amazonaws.com/prod/1559202/d3fd737e-97aa-11ee-b7ed-02a6bfeb93bd/2981514/a55eb826-60de-11f0-b35b-0a58a9feac02/file/25-26_Elementary_Handbook.pdf</t>
         </is>
       </c>
       <c r="H111" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I111" s="8" t="inlineStr">
@@ -24863,15 +24895,19 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.rcsd.ms/about-rcsd/school-board</t>
         </is>
       </c>
       <c r="H112" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I112" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I112" s="8" t="inlineStr">
+        <is>
+          <t>Held - official School Board page names only 4 of 5 trustees.</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="8" t="inlineStr">
@@ -24987,12 +25023,12 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.scott.k12.ms.us/apps/pages/index.jsp?uREC_ID=1349468&amp;type=d</t>
         </is>
       </c>
       <c r="H115" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I115" s="8" t="inlineStr"/>
@@ -25069,12 +25105,12 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://files-backend.assets.thrillshare.com/documents/asset/uploaded_file/5724/Scsd/c543a70a-8de3-4a14-803b-17f47a6c2589/ADOPTED_SCSD_Classified_Employee_Handbook_2025.pdf?disposition=inline</t>
         </is>
       </c>
       <c r="H117" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I117" s="8" t="inlineStr"/>
@@ -25110,12 +25146,12 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.smithcountyschools.net/smithcountyschoolboard</t>
         </is>
       </c>
       <c r="H118" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I118" s="8" t="inlineStr"/>
@@ -25156,12 +25192,12 @@
       </c>
       <c r="H119" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Roster held</t>
         </is>
       </c>
       <c r="I119" s="8" t="inlineStr">
         <is>
-          <t>Type unresolved — classification pass (Code provisos + local acts) Parent review: classification recorded as Elected on the OSA audit's elected-board language; legal type remains Unresolved (no official source states it).</t>
+          <t>Held - no official board roster published (district site has no board page).</t>
         </is>
       </c>
     </row>
@@ -25196,12 +25232,12 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://core-docs.s3.us-east-1.amazonaws.com/documents/asset/uploaded_file/5225/POS/4956030/2025_-_South_Panola_Schools_-_Pope_4-8_Handbook_v4.pdf</t>
         </is>
       </c>
       <c r="H120" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I120" s="8" t="inlineStr">
@@ -25241,17 +25277,17 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.southpike.org/apps/pages/index.jsp?uREC_ID=1763451&amp;type=d&amp;pREC_ID=1944756</t>
         </is>
       </c>
       <c r="H121" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Roster held</t>
         </is>
       </c>
       <c r="I121" s="8" t="inlineStr">
         <is>
-          <t>Type unresolved — classification pass (Code provisos + local acts) Parent review: classification recorded as Elected on the OSA audit's elected-board language; legal type remains Unresolved (no official source states it).</t>
+          <t>Held - board page appears stale (names a superseded superintendent); roster currency unconfirmed.</t>
         </is>
       </c>
     </row>
@@ -25286,12 +25322,12 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://southtippahschools.com/wp-content/uploads/2026/07/26-27-RES-Handbook.pdf</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I122" s="8" t="inlineStr">
@@ -25331,12 +25367,12 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.cityofstarkville.org/108/School-Board-of-Trustees</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I123" s="8" t="inlineStr"/>
@@ -25372,15 +25408,19 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://campussuite-storage.s3.amazonaws.com/prod/1558980/d120948e-19e5-11ea-a637-123223a58045/2135589/61ca20b4-d12d-11ea-bfce-0aeac43e6be1/file/20-21%20SCSD%20Student%20Handbook%20FINAL%20PDF.pdf</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I124" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I124" s="8" t="inlineStr">
+        <is>
+          <t>Held - only complete roster is the 2020-21 handbook and MDE's 2024 report names a president not on it; membership has changed.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="8" t="inlineStr">
@@ -25413,15 +25453,19 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://content.myconnectsuite.com/api/documents/eaa9ead837aa4c068a33e357d72e5d19</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I125" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I125" s="8" t="inlineStr">
+        <is>
+          <t>Held - newest roster found is the 2023-24 district calendar; may be stale.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="8" t="inlineStr">
@@ -25454,12 +25498,12 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://files-backend.assets.thrillshare.com/documents/asset/uploaded_file/5509/Tcs/45bd9226-a96a-4c99-9b4f-6dcc77ca5693/TCSD-Student-Handbook-2025-2026.pdf?disposition=inline</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I126" s="8" t="inlineStr"/>
@@ -25500,10 +25544,14 @@
       </c>
       <c r="H127" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
-        </is>
-      </c>
-      <c r="I127" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I127" s="8" t="inlineStr">
+        <is>
+          <t>Held - no official board roster published (district site, Simbli portal, handbooks checked).</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="8" t="inlineStr">
@@ -25536,15 +25584,19 @@
       </c>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://mdek12.org/communications/2022/11/10/state-board-appoints-tunica-county-school-district-advisory-board-members_20221110/</t>
         </is>
       </c>
       <c r="H128" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I128" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I128" s="8" t="inlineStr">
+        <is>
+          <t>Held - district publishes no roster; the 2022 MDE-appointed transitional board is the newest official list, and post-2024 election outcomes are unverified.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="8" t="inlineStr">
@@ -25622,12 +25674,12 @@
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://content.myconnectsuite.com/api/documents/fc0bacac4a2f466195f893b0c05708e5</t>
         </is>
       </c>
       <c r="H130" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I130" s="8" t="inlineStr"/>
@@ -25708,12 +25760,12 @@
       </c>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://vwsd-k12.community.highbond.com/document/b662c2d6-d8d5-4cc9-9a4c-e483270e96f7/</t>
         </is>
       </c>
       <c r="H132" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I132" s="8" t="inlineStr">
@@ -25753,12 +25805,12 @@
       </c>
       <c r="G133" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.wcsd.k12.ms.us/board</t>
         </is>
       </c>
       <c r="H133" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I133" s="8" t="inlineStr"/>
@@ -25839,12 +25891,12 @@
       </c>
       <c r="G135" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://files.smartsites.parentsquare.com/9515/regular_board_meeting_notice_9-25-25.pdf</t>
         </is>
       </c>
       <c r="H135" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I135" s="8" t="inlineStr"/>
@@ -25880,15 +25932,19 @@
       </c>
       <c r="G136" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://content.myconnectsuite.com/api/documents/7643ffd134314502b371798c2b5a3041.pdf</t>
         </is>
       </c>
       <c r="H136" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I136" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I136" s="8" t="inlineStr">
+        <is>
+          <t>Held - handbook roster appears stale (MDE's 2024 president is not among its five).</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="8" t="inlineStr">
@@ -25926,10 +25982,14 @@
       </c>
       <c r="H137" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I137" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I137" s="8" t="inlineStr">
+        <is>
+          <t>Held - no official board roster published (2026 agendas name no members).</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="8" t="inlineStr">
@@ -25962,12 +26022,12 @@
       </c>
       <c r="G138" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.westjasper.org/boe</t>
         </is>
       </c>
       <c r="H138" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I138" s="8" t="inlineStr"/>
@@ -26003,15 +26063,19 @@
       </c>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://content.myconnectsuite.com/api/documents/2aa8993f72e54458991c76e8bd6c6b9e.pdf</t>
         </is>
       </c>
       <c r="H139" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I139" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I139" s="8" t="inlineStr">
+        <is>
+          <t>Held - newest roster found is the district Strategic Plan revised July 2023; may be stale.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="8" t="inlineStr">
@@ -26090,12 +26154,12 @@
       </c>
       <c r="H141" s="8" t="inlineStr">
         <is>
-          <t>Classified — ready for roster pass</t>
+          <t>Roster held</t>
         </is>
       </c>
       <c r="I141" s="8" t="inlineStr">
         <is>
-          <t>Type unresolved — classification pass (Code provisos + local acts)</t>
+          <t>Held - no official roster published, and audits conflict on whether the board has five or six members.</t>
         </is>
       </c>
     </row>
@@ -26135,10 +26199,14 @@
       </c>
       <c r="H142" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I142" s="8" t="inlineStr"/>
+          <t>Deferred - District of Transformation</t>
+        </is>
+      </c>
+      <c r="I142" s="8" t="inlineStr">
+        <is>
+          <t>District of Transformation per MDE's official Jan. 15, 2026 news release: the elected local board is not functioning and the district is state-led. Deferred with the other Transformation districts.</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="8" t="inlineStr">
@@ -26171,12 +26239,12 @@
       </c>
       <c r="G143" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://files-backend.assets.thrillshare.com/documents/asset/uploaded_file/1202/Wmcsd/6d468a42-b49a-4aa8-9ee3-e72f0e66909e/WSS_Handbook_25-26.pdf?disposition=inline</t>
         </is>
       </c>
       <c r="H143" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I143" s="8" t="inlineStr"/>
@@ -26257,12 +26325,12 @@
       </c>
       <c r="G145" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://resources.finalsite.net/images/v1764607251/yazook12org/yktbf7afioba4gwqlpyx/YCSD2025-26EmployeeHandbook12.pdf</t>
         </is>
       </c>
       <c r="H145" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I145" s="8" t="inlineStr"/>

</xml_diff>

<commit_message>
MS #158: round-2 sheet update (5 more minted; Western Line + West Tallahatchie hold notes)
</commit_message>
<xml_diff>
--- a/reference/MS Rolling Audit/MS_Municipalities.xlsx
+++ b/reference/MS Rolling Audit/MS_Municipalities.xlsx
@@ -19814,7 +19814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="8" min="1" max="1"/>
@@ -20062,6 +20062,33 @@
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Boone</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Roster pass round 2 (issue #158): Walter supplied the official board-page URLs for five of the no-roster holds; all five were read firsthand and minted onto PR #161 (Copiah County, Greene County, South Delta, Tishomingo County SMSD, West Bolivar Consolidated) - 73 districts minted in total. South Delta's page names four members with the Vice-President cell blank as published (an MDE report naming a different president is flagged on its row); West Bolivar's page shows its fifth seat as VACANT. Walter also supplied Western Line and West Tallahatchie board pages: both were read and both remain held - Western Line's page shows six captioned photos (one captioned only 'McDavid', no seating labels, audits conflict 5 vs 6 members); West Tallahatchie's page has no text roster, only six photo alt-text names against a five-seat structure.</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>School Districts, Status Log</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>District board pages supplied by Walter 2026-10-16 (copiah.ms, gcsd.ms.gov, southdelta.k12.ms.us, tcsk12.com, wbcsdk12.org, westernline.org, wtsdschools.org)</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Boone</t>
         </is>
@@ -21284,17 +21311,17 @@
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.copiah.ms/school-board/index</t>
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
-          <t>Held - district site (www.copiah.ms) unreachable during capture; no official roster located.</t>
+          <t>Minted 2026-10-16 from the district's School Board page (URL supplied by Walter): five members, no seat labels published.</t>
         </is>
       </c>
     </row>
@@ -21796,17 +21823,17 @@
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.gcsd.ms.gov/school-board</t>
         </is>
       </c>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I40" s="8" t="inlineStr">
         <is>
-          <t>Held - district site returns no readable board page; no official roster located.</t>
+          <t>Minted 2026-10-16 from the district's School Board page at gcsd.ms.gov (URL supplied by Walter): five members, one per numbered district.</t>
         </is>
       </c>
     </row>
@@ -25187,17 +25214,17 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>http://www.southdelta.k12.ms.us/board-of-education/</t>
         </is>
       </c>
       <c r="H119" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I119" s="8" t="inlineStr">
         <is>
-          <t>Held - no official board roster published (district site has no board page).</t>
+          <t>Minted 2026-10-16 from the district's Board of Education page (URL supplied by Walter): four members named (Young, President; Grayson, Secretary; McClendon; Sias) and the Vice-President name cell is blank as published - the fifth seat is unnamed there. Flag: an MDE report located during the roster pass named a different president (John Evans); the district's own page was used and the discrepancy is recorded here.</t>
         </is>
       </c>
     </row>
@@ -25539,12 +25566,12 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.tcsk12.com/page/board-members</t>
         </is>
       </c>
       <c r="H127" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I127" s="8" t="inlineStr">
@@ -25977,17 +26004,17 @@
       </c>
       <c r="G137" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.wbcsdk12.org/trustees</t>
         </is>
       </c>
       <c r="H137" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I137" s="8" t="inlineStr">
         <is>
-          <t>Held - no official board roster published (2026 agendas name no members).</t>
+          <t>Minted 2026-10-16 from the district's Trustees page (URL supplied by Walter): four named trustees (Thomas, Bell, Lloyd, Tate) and the fifth seat shown as VACANT, as published.</t>
         </is>
       </c>
     </row>
@@ -26113,10 +26140,14 @@
       </c>
       <c r="H140" s="8" t="inlineStr">
         <is>
-          <t>Seeded — class rule</t>
-        </is>
-      </c>
-      <c r="I140" s="8" t="inlineStr"/>
+          <t>Roster held</t>
+        </is>
+      </c>
+      <c r="I140" s="8" t="inlineStr">
+        <is>
+          <t>Held - the district's official School Board page (wtsdschools.org/page/school-board, supplied by Walter 2026-10-16) publishes no text roster; its photo set names six people in image alt text (Marvin George, Gloria Carter, LaTrencia Bounds, Lucinda Berryhill, Sharon Bailey, Kelvin Pulley) with no roles or seats, and the count conflicts with the five-seat structure - one may be a non-member officer. Not minted until a labeled source appears.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="8" t="inlineStr">
@@ -26159,7 +26190,7 @@
       </c>
       <c r="I141" s="8" t="inlineStr">
         <is>
-          <t>Held - no official roster published, and audits conflict on whether the board has five or six members.</t>
+          <t>Held - the district's official School Board page (westernline.org/schoolboard, supplied by Walter 2026-10-16) shows six captioned member photos - Jamelda Fulton, Larry Franklin, Ruth Evans, Casandra Holiman, Greg Welch, and a sixth captioned only '/MCDAVID' - with no seat or elected/appointed labels. The six photos support the older audit's six-member structure (5 elected + 1 appointed) over the later audit's five elected, but the appointed member and the sixth member's full name cannot be identified from official sources, so memberships are not minted.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MS #158: rounds 3-4 sheet update (Western Line + West Tallahatchie minted; Western Line seats corrected to 6)
</commit_message>
<xml_diff>
--- a/reference/MS Rolling Audit/MS_Municipalities.xlsx
+++ b/reference/MS Rolling Audit/MS_Municipalities.xlsx
@@ -19814,7 +19814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="8" min="1" max="1"/>
@@ -20089,6 +20089,33 @@
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Boone</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roster pass rounds 3-4 (issue #158): Western Line and West Tallahatchie Consolidated minted onto PR #161 after Walter supplied the missing identifications - Western Line's sixth member is Norma McDavid and Casandra Holiman is its appointed member (six-member board, 5 elected + 1 appointed, Seats corrected to 6); West Tallahatchie's page labels its members by district (Berryhill D1, George D2, Carter D3, Bailey D4, Bounds D5) and Kelvin Pulley is its Board Attorney, not a member. 75 districts minted; 21 still held.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>School Districts, Status Log</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>District board pages (westernline.org, wtsdschools.org) with identifications supplied by Walter 2026-10-16</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>Boone</t>
         </is>
@@ -26135,17 +26162,17 @@
       </c>
       <c r="G140" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.wtsdschools.org/page/school-board</t>
         </is>
       </c>
       <c r="H140" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I140" s="8" t="inlineStr">
         <is>
-          <t>Held - the district's official School Board page (wtsdschools.org/page/school-board, supplied by Walter 2026-10-16) publishes no text roster; its photo set names six people in image alt text (Marvin George, Gloria Carter, LaTrencia Bounds, Lucinda Berryhill, Sharon Bailey, Kelvin Pulley) with no roles or seats, and the count conflicts with the five-seat structure - one may be a non-member officer. Not minted until a labeled source appears.</t>
+          <t>Minted 2026-10-16 from the district's School Board page as labeled there and confirmed by Walter: Berryhill (D1), George (D2), Carter (D3, Secretary), Bailey (D4, President), Bounds (D5). Kelvin Pulley appears in the same photo set as Board Attorney - not a member - which resolves the six-names-vs-five-seats conflict that held the district in round 2.</t>
         </is>
       </c>
     </row>
@@ -26171,7 +26198,7 @@
         </is>
       </c>
       <c r="E141" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F141" s="8" t="inlineStr">
         <is>
@@ -26180,17 +26207,17 @@
       </c>
       <c r="G141" s="8" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>https://www.westernline.org/schoolboard</t>
         </is>
       </c>
       <c r="H141" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I141" s="8" t="inlineStr">
         <is>
-          <t>Held - the district's official School Board page (westernline.org/schoolboard, supplied by Walter 2026-10-16) shows six captioned member photos - Jamelda Fulton, Larry Franklin, Ruth Evans, Casandra Holiman, Greg Welch, and a sixth captioned only '/MCDAVID' - with no seat or elected/appointed labels. The six photos support the older audit's six-member structure (5 elected + 1 appointed) over the later audit's five elected, but the appointed member and the sixth member's full name cannot be identified from official sources, so memberships are not minted.</t>
+          <t>Minted 2026-10-16: the district's School Board page shows six captioned member photos; Walter supplied the two identifications the page does not make - the member captioned only '/MCDAVID' is Norma McDavid, and Casandra Holiman is the board's appointed member. Six members: five elected + Holiman appointed (consistent with the older OSA audit's six-member structure).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MS #158: round-5 sheet update (Coffeeville, Jefferson, Lamar, Rankin minted; Oxford hold note)
</commit_message>
<xml_diff>
--- a/reference/MS Rolling Audit/MS_Municipalities.xlsx
+++ b/reference/MS Rolling Audit/MS_Municipalities.xlsx
@@ -19814,7 +19814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="8" min="1" max="1"/>
@@ -20095,27 +20095,54 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Roster pass rounds 3-4 (issue #158): Western Line and West Tallahatchie Consolidated minted onto PR #161 after Walter supplied the missing identifications - Western Line's sixth member is Norma McDavid and Casandra Holiman is its appointed member (six-member board, 5 elected + 1 appointed, Seats corrected to 6); West Tallahatchie's page labels its members by district (Berryhill D1, George D2, Carter D3, Bailey D4, Bounds D5) and Kelvin Pulley is its Board Attorney, not a member. 75 districts minted; 21 still held.</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>School Districts, Status Log</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>District board pages (westernline.org, wtsdschools.org) with identifications supplied by Walter 2026-10-16</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Boone</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Roster pass round 5 (issue #158): Coffeeville, Jefferson County, Lamar County, and Rankin County minted onto PR #161 from rosters Walter supplied (Coffeeville's fifth trustee is Linda Bland; Jefferson's five completed by David Hamlin Jr. and Michael Malone; Lamar's District D confirmed vacant - post minted unfilled; Rankin's four trustees include its president, published as Grumpy Farmer). Oxford remains held: its members are now known, but as a Mixed board it still needs a source labeling which members are elected vs. appointed. 79 districts minted; 17 still held.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>School Districts, Status Log</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Board rosters supplied by Walter 2026-10-16</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Boone</t>
         </is>
@@ -21212,12 +21239,12 @@
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>Held - district board page names only 4 of 5 trustees; fifth member not named in any official source found.</t>
+          <t>Minted 2026-10-16: full five trustees confirmed by Walter - Polk (President), Steen (Vice President), Alisia Bland (Secretary), Townes (Parliamentarian), Linda Bland (Parent Liaison); Superintendent Dexter Green is not a member. No seat labels published.</t>
         </is>
       </c>
     </row>
@@ -22596,12 +22623,12 @@
       </c>
       <c r="H57" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I57" s="8" t="inlineStr">
         <is>
-          <t>Held - official board page names only 3 of 5 members.</t>
+          <t>Minted 2026-10-16: five members confirmed by Walter - Carolyn Smith (President), Claudine Middleton (Vice President), Kimberly Reed-Hutcherson (Executive Secretary), David Hamlin Jr., Michael Malone. The roster pass had found only the first three named. No seat labels published.</t>
         </is>
       </c>
     </row>
@@ -22926,12 +22953,12 @@
       </c>
       <c r="H65" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I65" s="8" t="inlineStr">
         <is>
-          <t>Held - official board page names 4 of 5 members; District D shown as an unnamed placeholder.</t>
+          <t>Minted 2026-10-16: Farmer (District A), Carlisle (B), Slade (C), Hensarling (E); District D confirmed vacant by Walter - the post is minted with no membership.</t>
         </is>
       </c>
     </row>
@@ -24304,7 +24331,7 @@
       </c>
       <c r="I97" s="8" t="inlineStr">
         <is>
-          <t>Held - official Board Members page lists only 4 of 5 members.</t>
+          <t>Held - Mixed board. The members are now known (Walter, 2026-10-16: Carter Myers, President; Lolita Gregory; Denson Hollis; Jordan Russell - with Paul Watkins as Board Attorney and Ashley Wilkinson as Board Secretary, both staff), but no official source labels which members hold the elected added-territory seats vs. the appointed seats, so memberships cannot be minted without guessing. A source labeling the members (or Walter's identification, as with Western Line) unblocks it.</t>
         </is>
       </c>
     </row>
@@ -24954,12 +24981,12 @@
       </c>
       <c r="H112" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I112" s="8" t="inlineStr">
         <is>
-          <t>Held - official School Board page names only 4 of 5 trustees.</t>
+          <t>Minted 2026-10-16: four trustees confirmed by Walter - Grumpy Farmer (President; published name, confirmed by Walter), David Dyess (Vice President), Tommy McCarver, Katherine McKinion (page form 'Katherine (Liza) McKinion'). Fred Harrell (Attorney) and Kym Jamison (Secretary) are staff roles, not members. The fifth seat is not named on the page.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MS #158: Oxford hold note refined (Russell confirmed appointed; 3A+2E structure documented)
</commit_message>
<xml_diff>
--- a/reference/MS Rolling Audit/MS_Municipalities.xlsx
+++ b/reference/MS Rolling Audit/MS_Municipalities.xlsx
@@ -20122,27 +20122,27 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Roster pass round 5 (issue #158): Coffeeville, Jefferson County, Lamar County, and Rankin County minted onto PR #161 from rosters Walter supplied (Coffeeville's fifth trustee is Linda Bland; Jefferson's five completed by David Hamlin Jr. and Michael Malone; Lamar's District D confirmed vacant - post minted unfilled; Rankin's four trustees include its president, published as Grumpy Farmer). Oxford remains held: its members are now known, but as a Mixed board it still needs a source labeling which members are elected vs. appointed. 79 districts minted; 17 still held.</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>School Districts, Status Log</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Board rosters supplied by Walter 2026-10-16</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>Boone</t>
         </is>
@@ -24331,7 +24331,7 @@
       </c>
       <c r="I97" s="8" t="inlineStr">
         <is>
-          <t>Held - Mixed board. The members are now known (Walter, 2026-10-16: Carter Myers, President; Lolita Gregory; Denson Hollis; Jordan Russell - with Paul Watkins as Board Attorney and Ashley Wilkinson as Board Secretary, both staff), but no official source labels which members hold the elected added-territory seats vs. the appointed seats, so memberships cannot be minted without guessing. A source labeling the members (or Walter's identification, as with Western Line) unblocks it.</t>
+          <t>Held - Mixed board (5 seats: 3 appointed by the City of Oxford + 2 elected, per the city's official minute Book 34). Jordan Russell is confirmed APPOINTED (the district's own welcome post says he joined 'following his appointment'; confirmed by Walter 2026-10-16). The other current members - Carter Myers (President), Lolita Gregory, Denson Hollis - are unlabeled, the board page currently lists only four members, and Ashley Wilkinson's status is ambiguous (directory lists her as Board Secretary apart from the members, but Gregory attested the Sept. 22, 2025 board resolution as Board Secretary, and classification research noted a Nov. 2022 trustee election involving 'Reed/Wilkinson'). Remaining need: which two of the remaining seats are the elected ones and who holds them - a labeling source or Walter's identification unblocks it, as with Western Line.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MS #158: Poplarville minted as appointed holdovers (board converted to elected eff. 2026-07-01)
</commit_message>
<xml_diff>
--- a/reference/MS Rolling Audit/MS_Municipalities.xlsx
+++ b/reference/MS Rolling Audit/MS_Municipalities.xlsx
@@ -19814,7 +19814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="8" min="1" max="1"/>
@@ -20143,6 +20143,33 @@
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Boone</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Poplarville Special Municipal Separate added in a follow-up PR to #161 (issue #158; PR #161 was merged while this addition was in build, so it landed separately): its classification flag resolved - the Pearl River County Board of Supervisors adopted Poplarville School Board Election Districts effective July 1, 2026, converting the board from appointed to elected (first election Nov. 3, 2026, three of five seats). On Walter's decision it was minted now as appointed holdovers: the five current trustees (Smith, Houston, Miller, Jordan, Johnson) recorded how_seated appointed on a single five-seat post (no district assignments published). Citation caution recorded on the row: the 'House Bill 1142' named in the county post and press is an unrelated bench-warrant bill and is not cited. 80 districts minted; Poplarville's Nov. 3 winners to follow after the election.</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>School Districts, Status Log</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Pearl River County Board of Supervisors post (2026-05-04, pearlrivercounty.net); Poplarville SD Board of Trustees page (poplarvilleschools.org)</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>Boone</t>
         </is>
@@ -24791,7 +24818,7 @@
       </c>
       <c r="D108" s="8" t="inlineStr">
         <is>
-          <t>Appointed</t>
+          <t>Elected</t>
         </is>
       </c>
       <c r="E108" s="8" t="n">
@@ -24799,22 +24826,22 @@
       </c>
       <c r="F108" s="8" t="inlineStr">
         <is>
-          <t>OSA FY2023 audit Note 1 states the district is a related organization of the city of Poplarville because the city's governing authority selects a majority of the board (appointments split between the Board of Aldermen and the Pearl River County Board of Supervisors; five-member board). Picayune Item reports in May-June 2026 claim a 2026 law makes all five seats elected effective July 1, 2026, but the cited bill number is garbled in the article and no official act text or district announcement was located, so the last officially evidenced status (appointed) is recorded. [https://www.osa.ms.gov/sites/default/files/2024-08/23sPoplarville%2520School%2520District-cpa.pdf]</t>
+          <t>Resolved 2026-10-16: the Pearl River County Board of Supervisors (official county post, May 4, 2026) adopted Poplarville School Board Election Districts effective July 1, 2026, converting all five trustee seats from appointed to elected (five single-member districts; staggered terms, three seats in midterm years and two in presidential years; first election Nov. 3, 2026). The county post and press reports name 'House Bill 1142,' but the official 2026 HB 1142 is an unrelated bench-warrant bill, so that bill number is not cited. Supersedes the FY2023 OSA audit Note 1 (appointed; related organization of the city). [https://pearlrivercounty.net/m/newsflash/home/detail/42]</t>
         </is>
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>Not applicable (appointed board)</t>
+          <t>https://poplarvilleschools.org/?p=907168</t>
         </is>
       </c>
       <c r="H108" s="8" t="inlineStr">
         <is>
-          <t>Classified — out of scope (appointed)</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I108" s="8" t="inlineStr">
         <is>
-          <t>FLAG: 2026 newspaper reports claim a 2026 law makes all five trustees elected effective July 1, 2026 (first election Nov. 2026), but the bill citation is garbled and no official act text was found — re-check the 2026 local-and-private legislation before the November 2026 election; classification rests on the last official evidence (FY2023 OSA audit).</t>
+          <t>Minted 2026-10-16 as appointed holdovers in a follow-up PR (PR #161 merged while the addition was being built) (Walter's decision, 2026-10-16): the five current trustees - Smith (President), Houston (Vice President), Miller (Secretary), Jordan, Johnson - were seated by appointment under the prior system and are recorded how_seated appointed; the district publishes no district assignments for them, so a single five-seat post is used. The Nov. 3, 2026 winners are to be seated by a follow-up build.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MS #158: tracking sheet - 7 holdovers minted; West Point re-held as unlabeled Mixed (classification conflict flagged); Enterprise/North Bolivar rechecked
</commit_message>
<xml_diff>
--- a/reference/MS Rolling Audit/MS_Municipalities.xlsx
+++ b/reference/MS Rolling Audit/MS_Municipalities.xlsx
@@ -25,7 +25,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="9">
     <font>
       <name val="Calibri"/>
@@ -137,7 +139,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -188,6 +190,7 @@
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -20149,29 +20152,22 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Poplarville Special Municipal Separate added in a follow-up PR to #161 (issue #158; PR #161 was merged while this addition was in build, so it landed separately): its classification flag resolved - the Pearl River County Board of Supervisors adopted Poplarville School Board Election Districts effective July 1, 2026, converting the board from appointed to elected (first election Nov. 3, 2026, three of five seats). On Walter's decision it was minted now as appointed holdovers: the five current trustees (Smith, Houston, Miller, Jordan, Johnson) recorded how_seated appointed on a single five-seat post (no district assignments published). Citation caution recorded on the row: the 'House Bill 1142' named in the county post and press is an unrelated bench-warrant bill and is not cited. 80 districts minted; Poplarville's Nov. 3 winners to follow after the election.</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>School Districts, Status Log</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Pearl River County Board of Supervisors post (2026-05-04, pearlrivercounty.net); Poplarville SD Board of Trustees page (poplarvilleschools.org)</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Boone</t>
+      <c r="A13" s="18" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>School Districts</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Follow-up sweep (post-#161)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>7 holdovers minted (Neshoba conflict decided for Butler; Marshall, South Pike, Stone, Sunflower, Tunica, Webster on current live rosters). West Point re-held as unlabeled Mixed (live page states 2 elected + 3 city-appointed - conflicts with Elected classification; flagged). Enterprise and North Bolivar re-checked, still no current roster.</t>
         </is>
       </c>
     </row>
@@ -21664,7 +21660,7 @@
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>Held - only published roster is headed '2022-2023 School Year'; may be stale.</t>
+          <t>Rechecked 2026-10-16: the district's live School Board page still carries the 2022-2023 roster (Culbreth, Ivy, Kersh, Mosley, Freeman); the current handbook link is dead and no minutes or agendas are posted. Still held - no current official roster.</t>
         </is>
       </c>
     </row>
@@ -23524,17 +23520,17 @@
       </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
-          <t>https://www.marshallcountysd.org/article/909674</t>
+          <t>https://www.marshallcountysd.org/o/mcsd/page/board-of-education</t>
         </is>
       </c>
       <c r="H78" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I78" s="8" t="inlineStr">
         <is>
-          <t>Held - newest official roster found is a district article dated Nov 15, 2022; may be stale.</t>
+          <t>Current roster found on the district's live board page (2025-26 news): Hale (President), King (VP), Bryson (Secretary), Elizabeth Jones, Lee Seals. No complete seat labeling (Jones's bio cites District Two only), so minted on a single five-seat post.</t>
         </is>
       </c>
     </row>
@@ -23824,17 +23820,17 @@
       </c>
       <c r="G85" s="8" t="inlineStr">
         <is>
-          <t>https://files.smartsites.parentsquare.com/5429/employee_handbook_2025-2026_for_website.pdf</t>
+          <t>https://files.smartsites.parentsquare.com/5429/employee_handbook_2026-2027_final_for_website_1.pdf</t>
         </is>
       </c>
       <c r="H85" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I85" s="8" t="inlineStr">
         <is>
-          <t>Held - district 2025-26 handbook and county supervisors page conflict on the District Two member (Nicholson vs. Butler); needs verification.</t>
+          <t>Conflict resolved: the district's 2026-2027 Employee Handbook (p. 3) names Trent Butler for District Two, superseding the 2025-2026 handbook's Mary Ann Nicholson; the county supervisors page also names Butler. Full roster minted per-seat: Holley D1, Butler D2, Joyner D3, Waddell D4, Byars D5. Robert Lee Thomas is Attorney, not a member.</t>
         </is>
       </c>
     </row>
@@ -24051,7 +24047,7 @@
       </c>
       <c r="I90" s="8" t="inlineStr">
         <is>
-          <t>Held - newest roster located may be stale (district board page publishes agendas only).</t>
+          <t>Rechecked 2026-10-16: the board page publishes only a 2024-2025 calendar and agendas, no roster. The 2025-2026 Instructional Management Plan confirms Jefferick Butler is still board president, but the other four members are unconfirmed past the 2023-2024 handbook. Still held.</t>
         </is>
       </c>
     </row>
@@ -24818,7 +24814,7 @@
       </c>
       <c r="D108" s="8" t="inlineStr">
         <is>
-          <t>Elected</t>
+          <t>Appointed</t>
         </is>
       </c>
       <c r="E108" s="8" t="n">
@@ -24826,22 +24822,22 @@
       </c>
       <c r="F108" s="8" t="inlineStr">
         <is>
-          <t>Resolved 2026-10-16: the Pearl River County Board of Supervisors (official county post, May 4, 2026) adopted Poplarville School Board Election Districts effective July 1, 2026, converting all five trustee seats from appointed to elected (five single-member districts; staggered terms, three seats in midterm years and two in presidential years; first election Nov. 3, 2026). The county post and press reports name 'House Bill 1142,' but the official 2026 HB 1142 is an unrelated bench-warrant bill, so that bill number is not cited. Supersedes the FY2023 OSA audit Note 1 (appointed; related organization of the city). [https://pearlrivercounty.net/m/newsflash/home/detail/42]</t>
+          <t>OSA FY2023 audit Note 1 states the district is a related organization of the city of Poplarville because the city's governing authority selects a majority of the board (appointments split between the Board of Aldermen and the Pearl River County Board of Supervisors; five-member board). Picayune Item reports in May-June 2026 claim a 2026 law makes all five seats elected effective July 1, 2026, but the cited bill number is garbled in the article and no official act text or district announcement was located, so the last officially evidenced status (appointed) is recorded. [https://www.osa.ms.gov/sites/default/files/2024-08/23sPoplarville%2520School%2520District-cpa.pdf]</t>
         </is>
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>https://poplarvilleschools.org/?p=907168</t>
+          <t>Not applicable (appointed board)</t>
         </is>
       </c>
       <c r="H108" s="8" t="inlineStr">
         <is>
-          <t>Minted</t>
+          <t>Classified — out of scope (appointed)</t>
         </is>
       </c>
       <c r="I108" s="8" t="inlineStr">
         <is>
-          <t>Minted 2026-10-16 as appointed holdovers in a follow-up PR (PR #161 merged while the addition was being built) (Walter's decision, 2026-10-16): the five current trustees - Smith (President), Houston (Vice President), Miller (Secretary), Jordan, Johnson - were seated by appointment under the prior system and are recorded how_seated appointed; the district publishes no district assignments for them, so a single five-seat post is used. The Nov. 3, 2026 winners are to be seated by a follow-up build.</t>
+          <t>FLAG: 2026 newspaper reports claim a 2026 law makes all five trustees elected effective July 1, 2026 (first election Nov. 2026), but the bill citation is garbled and no official act text was found — re-check the 2026 local-and-private legislation before the November 2026 election; classification rests on the last official evidence (FY2023 OSA audit).</t>
         </is>
       </c>
     </row>
@@ -25390,12 +25386,12 @@
       </c>
       <c r="H121" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I121" s="8" t="inlineStr">
         <is>
-          <t>Held - board page appears stale (names a superseded superintendent); roster currency unconfirmed.</t>
+          <t>Current roster on the district's live board page alongside the 2026-27 handbook; current superintendent (Holmes) named, so the earlier staleness concern is resolved. Andrews, Brumfield, Christian, Lampton, Martin; no labels printed - single five-seat post. Lem Mitchell is Board Attorney, excluded.</t>
         </is>
       </c>
     </row>
@@ -25516,17 +25512,17 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>https://campussuite-storage.s3.amazonaws.com/prod/1558980/d120948e-19e5-11ea-a637-123223a58045/2135589/61ca20b4-d12d-11ea-bfce-0aeac43e6be1/file/20-21%20SCSD%20Student%20Handbook%20FINAL%20PDF.pdf</t>
+          <t>https://www.stoneschools.org/about/school-board</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I124" s="8" t="inlineStr">
         <is>
-          <t>Held - only complete roster is the 2020-21 handbook and MDE's 2024 report names a president not on it; membership has changed.</t>
+          <t>Current labeled roster on the district's live board page, superseding the 2020-21 handbook: Schuman (President) D1, Dedeaux D2, Main D3, Wegner D4, Bond D5. Sean Courtney is Attorney, excluded.</t>
         </is>
       </c>
     </row>
@@ -25561,17 +25557,17 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>https://content.myconnectsuite.com/api/documents/eaa9ead837aa4c068a33e357d72e5d19</t>
+          <t>https://www.sunflower.k12.ms.us/aboutboe</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I125" s="8" t="inlineStr">
         <is>
-          <t>Held - newest roster found is the 2023-24 district calendar; may be stale.</t>
+          <t>Current labeled roster on the district's live board page: Johnson (President) D3, Sibley (VP) D1, Townsend (Secretary) D5, Kimbrough D2, Norwood D4. Disclosure: the page prints Johnson's term expiring 12/2025 while listing her as sitting President; the SOS Nov 4, 2025 special county postings carry no Sunflower trustee filing or successor, so the roster is recorded as published.</t>
         </is>
       </c>
     </row>
@@ -25692,17 +25688,17 @@
       </c>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t>https://mdek12.org/communications/2022/11/10/state-board-appoints-tunica-county-school-district-advisory-board-members_20221110/</t>
+          <t>https://www.tunicak12.org/about-us/board-of-education</t>
         </is>
       </c>
       <c r="H128" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I128" s="8" t="inlineStr">
         <is>
-          <t>Held - district publishes no roster; the 2022 MDE-appointed transitional board is the newest official list, and post-2024 election outcomes are unverified.</t>
+          <t>Current labeled roster on the district's live board page (Jan-Jun 2026 agendas posted): Hall D1, Johnson (VP) D2, Gill D3, Autry D4, Matthews D5. This is the ELECTED successor board: a Tunica County Election Commission order of Sept 23, 2025, posted by the SOS, declares Hall and Matthews elected without opposition in Nov 2025; D2-D4 hold staggered terms.</t>
         </is>
       </c>
     </row>
@@ -26040,17 +26036,17 @@
       </c>
       <c r="G136" s="8" t="inlineStr">
         <is>
-          <t>https://content.myconnectsuite.com/api/documents/7643ffd134314502b371798c2b5a3041.pdf</t>
+          <t>https://www.webstercountyschools.org/schoolboard</t>
         </is>
       </c>
       <c r="H136" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I136" s="8" t="inlineStr">
         <is>
-          <t>Held - handbook roster appears stale (MDE's 2024 president is not among its five).</t>
+          <t>Current roster on the district's live board page (links 2025-26 and 2026-27 meeting dates), superseding the stale handbook roster: Bingham, Davis, Hood, King, Palmer. No labels printed - single five-seat post.</t>
         </is>
       </c>
     </row>
@@ -26181,7 +26177,7 @@
       </c>
       <c r="I139" s="8" t="inlineStr">
         <is>
-          <t>Held - newest roster found is the district Strategic Plan revised July 2023; may be stale.</t>
+          <t>Rechecked 2026-10-16: the district's live board page publishes a current roster (Gene Brown, Chairman; Tommy Coleman, Vice-Chairman; Laquante Pruitt, Secretary; Israel Lee; Trina Davidson) - BUT the same page states two members are elected by voters outside the city limits and three are selected by the City of West Point's governing authorities, i.e. a MIXED board, which conflicts with this sheet's Elected classification. Members carry no per-member labels. HELD as an unlabeled Mixed board; classification conflict flagged for Walter 2026-10-16.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MS #158: tracking sheet - Ocean Springs/Pass Christian minted; Oxford, New Albany, Picayune, Pontotoc City, Canton hold notes updated with partial labels
</commit_message>
<xml_diff>
--- a/reference/MS Rolling Audit/MS_Municipalities.xlsx
+++ b/reference/MS Rolling Audit/MS_Municipalities.xlsx
@@ -19817,7 +19817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="8" min="1" max="1"/>
@@ -20155,19 +20155,39 @@
       <c r="A13" s="18" t="n">
         <v>46311</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>School Districts</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Follow-up sweep (post-#161)</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>7 holdovers minted (Neshoba conflict decided for Butler; Marshall, South Pike, Stone, Sunflower, Tunica, Webster on current live rosters). West Point re-held as unlabeled Mixed (live page states 2 elected + 3 city-appointed - conflicts with Elected classification; flagged). Enterprise and North Bolivar re-checked, still no current roster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>School Districts</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Mixed-board labeling sweep</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Ocean Springs and Pass Christian resolved and minted (elected seats proven by certified county recapitulations; appointed seats on the official structures). Oxford narrowed to one unknown (Wilkinson elected 2022; Hollis and Russell appointed; Myers-vs-Gregory blocked on corrupted City Minute Book 124). New Albany 2/5, Picayune 1/5, Pontotoc City 2/5 labeled; Canton mechanism documented, members unlabeled.</t>
         </is>
       </c>
     </row>
@@ -20848,7 +20868,7 @@
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>Held - roster lists 5 trustees but publishes no per-member elected/appointed labels for this Mixed board, and the page may lag current membership; needs a source labeling each member.</t>
+          <t>Held - mechanism documented, no current member labeled (2026-10-16). Glen Lacey's seat is an APPOINTED seat: district special-call minutes, Mar 6, 2026, address filling the vacancy from the expiration of Lacey's term, and a City of Canton agenda (Mar 3, 2026) carries a school-board appointment item for the term March 2026-February 2031 (appointee name blank in the posted agenda). Current members Johnny Brown, Lenderrick Taylor, Peter Brown, Jacqueline Griffin, Kimberly Lott carry no labels in any reachable official record; no Canton trustee contest appears in SOS Madison County recaps 2019-2025. Minutes Jan-May 2026 list only four members at times (Lott's accession is undocumented).</t>
         </is>
       </c>
     </row>
@@ -23920,7 +23940,7 @@
       </c>
       <c r="I87" s="8" t="inlineStr">
         <is>
-          <t>Held - Mixed board; district page lists all five trustees with no elected/appointed labels; needs a labeling source.</t>
+          <t>Held - 2 of 5 labeled (2026-10-16). David Rainey ELECTED (Union County Election Commissioners order, Sept 13, 2021 - sole qualified candidate for the Added Territory seat; election dispensed with). Mark Garrett APPOINTED (district post, Aug 19, 2019 - appointed to Brad Clayton's unexpired term; no later election record found). Lauren Bailey, Cassie Henson, Barbara Washington unlabeled; no official source states the board's elected/appointed split (only one added-territory seat appears in SOS Union records 2016-2025).</t>
         </is>
       </c>
     </row>
@@ -24254,17 +24274,17 @@
       </c>
       <c r="G95" s="8" t="inlineStr">
         <is>
-          <t>https://www.ossdms.org/discoverossd/school-board-policies</t>
+          <t>https://oceansprings-ms.gov/304/Ocean-Springs-School-Board</t>
         </is>
       </c>
       <c r="H95" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I95" s="8" t="inlineStr">
         <is>
-          <t>Held - Mixed board; district page gives no per-member elected/appointed labels; needs a labeling source.</t>
+          <t>RESOLVED 2026-10-16: City of Ocean Springs school-board page states the structure (Board of Aldermen appoints 3; the other two are elected), corroborated by the OSA FY2023 audit. Elected proven by Jackson County Official Recapitulations: Tomaszewski (Nov 2, 2021 OSAT race) and Waters (Nov 5, 2024 OSAT race). Tiblier, Ronald Chambers ('Ron' on the district page), and Denyer hold the appointed seats on that structure. Minted as two posts (elected 2 / appointed 3).</t>
         </is>
       </c>
     </row>
@@ -24354,7 +24374,7 @@
       </c>
       <c r="I97" s="8" t="inlineStr">
         <is>
-          <t>Held - Mixed board (5 seats: 3 appointed by the City of Oxford + 2 elected, per the city's official minute Book 34). Jordan Russell is confirmed APPOINTED (the district's own welcome post says he joined 'following his appointment'; confirmed by Walter 2026-10-16). The other current members - Carter Myers (President), Lolita Gregory, Denson Hollis - are unlabeled, the board page currently lists only four members, and Ashley Wilkinson's status is ambiguous (directory lists her as Board Secretary apart from the members, but Gregory attested the Sept. 22, 2025 board resolution as Board Secretary, and classification research noted a Nov. 2022 trustee election involving 'Reed/Wilkinson'). Remaining need: which two of the remaining seats are the elected ones and who holds them - a labeling source or Walter's identification unblocks it, as with Western Line. Walter (2026-10-16): leave as follow-up research - not a blocker on issue #158.</t>
+          <t>Held - narrowed to ONE unknown (2026-10-16). Wilkinson question ANSWERED: Ashley Wilkinson IS the fifth trustee and is ELECTED - SOS Lafayette County Official Recapitulation, Nov 8, 2022 (Wilkinson 1,772 def. Romana Reed 996); oath Jan 23, 2023. 'Board Secretary' is an officer post the trustees elect among themselves (Gregory held it in 2025-26; Wilkinson holds it now; the staff clerk is LaTeasha Blackmon). Denson Hollis is APPOINTED (district post, Mar 25, 2025 - he sought the seat from the Mayor and Board of Aldermen; sworn in Mar 24, 2025). Jordan Russell is APPOINTED (oath Apr 13, 2026). Remaining unknown: which of Carter B. Myers (President) and Lolita Gregory holds the second elected seat - no election or appointment record for either found in SOS Lafayette recaps 2018-2024 or OSD minutes 2020-2026; the City of Oxford Minute Book 124 (Feb-Mar 2023, covering Gregory's accession) is a corrupted 123 MB file on the city's server and unreadable past its first segment. Walter (2026-10-16): follow-up research, not a blocker on #158.</t>
         </is>
       </c>
     </row>
@@ -24439,12 +24459,12 @@
       </c>
       <c r="H99" s="8" t="inlineStr">
         <is>
-          <t>Roster held</t>
+          <t>Minted</t>
         </is>
       </c>
       <c r="I99" s="8" t="inlineStr">
         <is>
-          <t>Held - Mixed board; district page gives no per-member elected/appointed labels; needs a labeling source.</t>
+          <t>RESOLVED 2026-10-16: Elected proven by certified Harrison County records - King (Election Commission certification, Sept 13, 2021) and Fortenberry (Official Recapitulation, Nov 5, 2024). Kalif appointed (city BOA minutes Nov 19, 2024: reappointed to a term ending Mar 31, 2030). Powell appointed by term-match to the city's Mar 2024 appointment process (naming vote in unposted Mar 27, 2024 minutes). Daniels appointed by elimination (both elected seats proven held; her term runs on the appointed March cycle). Minted as two posts (elected 2 / appointed 3) with the full reasoning in the source notes.</t>
         </is>
       </c>
     </row>
@@ -24706,7 +24726,7 @@
       </c>
       <c r="I105" s="8" t="inlineStr">
         <is>
-          <t>Held - Mixed board; district page gives no per-member elected/appointed labels; needs a labeling source.</t>
+          <t>Held - 1 of 5 labeled (2026-10-16). Structure documented in district Policy ABCD: one or two members are residents of the added territory and elected by its electors; the remaining members are chosen by majority vote of the City Council at its February meeting. Jake Smith ELECTED (Pearl River County, Nov 2, 2021 - sole candidate for 'Picayune School Board 1 Outside', term 2022-2026, declared elected under 23-15-839). No second Outside-seat election appears in 2020-2025 county records, but the current 1-vs-2 elected split is not officially stated and no council selection records could be retrieved (city site served no content). Robertson, Myers, Sweet, Bolden unlabeled.</t>
         </is>
       </c>
     </row>
@@ -24751,7 +24771,7 @@
       </c>
       <c r="I106" s="8" t="inlineStr">
         <is>
-          <t>Held - Mixed board; district page gives no per-member elected/appointed labels; needs a labeling source.</t>
+          <t>Held - 2 of 5 labeled (2026-10-16). Gaye Howard ELECTED (won the Municipal Separate School Board Member race, Pontotoc County General Elections Nov 3, 2020 and Nov 5, 2024, sole candidate both times). Benjamin Hill ELECTED (sole candidate, School District 6-Municipal Separate Trustee race, Nov 7, 2023). Phyllis High, Shane Clayton, Chase Jefcoat unlabeled - no election or appointment record found; no official source states the split (OSA FY2025 Note 1 'city selects a majority' is not decisive alone). City aldermen minutes unreachable.</t>
         </is>
       </c>
     </row>

</xml_diff>